<commit_message>
feat(orcamento): modelo v3 com FRETE (B38, lista CIF/FOB) e coluna R DESCRIÇÃO NO DAV
Editado pelo XML para manter as listas suspensas x14. Os blocos ITEM 1..27 descem uma linha; nada lia essas linhas. A B38 e a R2:R25 ficam desbloqueadas na aba protegida.
</commit_message>
<xml_diff>
--- a/orcamento/modelo/PLANILHA-BASE-v3.xlsx
+++ b/orcamento/modelo/PLANILHA-BASE-v3.xlsx
@@ -5963,7 +5963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI683"/>
+  <dimension ref="A1:BI684"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.7109375" style="1" customWidth="1"/>
@@ -5976,10 +5976,12 @@
     <col min="8" max="8" width="13.140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="22.85546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="26.28515625" style="2" customWidth="1"/>
-    <col min="11" max="61" width="14" style="3" customWidth="1"/>
+    <col min="11" max="17" width="14" style="3" customWidth="1"/>
+    <col min="18" max="18" width="45" style="3" customWidth="1"/>
+    <col min="19" max="61" width="14" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -6031,8 +6033,13 @@
       <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>DESCRIÇÃO NO DAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
       <c r="B2" s="7">
         <v>1</v>
@@ -6063,8 +6070,9 @@
       <c r="O2" s="35"/>
       <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
-    </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R2" s="35"/>
+    </row>
+    <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14"/>
       <c r="B3" s="7">
         <v>1</v>
@@ -6095,8 +6103,9 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
       <c r="Q3" s="12"/>
-    </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R3" s="12"/>
+    </row>
+    <row r="4" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14"/>
       <c r="B4" s="7">
         <v>1</v>
@@ -6127,8 +6136,9 @@
       <c r="O4" s="12"/>
       <c r="P4" s="12"/>
       <c r="Q4" s="12"/>
-    </row>
-    <row r="5" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R4" s="12"/>
+    </row>
+    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14"/>
       <c r="B5" s="7">
         <v>1</v>
@@ -6159,8 +6169,9 @@
       <c r="O5" s="12"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
-    </row>
-    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R5" s="12"/>
+    </row>
+    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15"/>
       <c r="B6" s="7">
         <v>1</v>
@@ -6191,8 +6202,9 @@
       <c r="O6" s="12"/>
       <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
-    </row>
-    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R6" s="12"/>
+    </row>
+    <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="7">
         <v>1</v>
@@ -6223,8 +6235,9 @@
       <c r="O7" s="12"/>
       <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
-    </row>
-    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R7" s="12"/>
+    </row>
+    <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="7">
         <v>1</v>
@@ -6255,8 +6268,9 @@
       <c r="O8" s="12"/>
       <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
-    </row>
-    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="7">
         <v>1</v>
@@ -6287,8 +6301,9 @@
       <c r="O9" s="12"/>
       <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
-    </row>
-    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R9" s="12"/>
+    </row>
+    <row r="10" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="7">
         <v>1</v>
@@ -6319,8 +6334,9 @@
       <c r="O10" s="12"/>
       <c r="P10" s="12"/>
       <c r="Q10" s="12"/>
-    </row>
-    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="7">
         <v>1</v>
@@ -6351,8 +6367,9 @@
       <c r="O11" s="12"/>
       <c r="P11" s="12"/>
       <c r="Q11" s="12"/>
-    </row>
-    <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R11" s="12"/>
+    </row>
+    <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="7">
         <v>1</v>
@@ -6383,8 +6400,9 @@
       <c r="O12" s="12"/>
       <c r="P12" s="12"/>
       <c r="Q12" s="12"/>
-    </row>
-    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="7">
         <v>1</v>
@@ -6415,8 +6433,9 @@
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
       <c r="Q13" s="12"/>
-    </row>
-    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R13" s="12"/>
+    </row>
+    <row r="14" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="7">
         <v>1</v>
@@ -6447,8 +6466,9 @@
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
       <c r="Q14" s="12"/>
-    </row>
-    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="7">
         <v>1</v>
@@ -6479,8 +6499,9 @@
       <c r="O15" s="12"/>
       <c r="P15" s="12"/>
       <c r="Q15" s="12"/>
-    </row>
-    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R15" s="12"/>
+    </row>
+    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" s="7">
         <v>1</v>
@@ -6511,8 +6532,9 @@
       <c r="O16" s="12"/>
       <c r="P16" s="12"/>
       <c r="Q16" s="12"/>
-    </row>
-    <row r="17" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="7">
         <v>1</v>
@@ -6543,8 +6565,9 @@
       <c r="O17" s="12"/>
       <c r="P17" s="12"/>
       <c r="Q17" s="12"/>
-    </row>
-    <row r="18" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R17" s="12"/>
+    </row>
+    <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="7">
         <v>1</v>
@@ -6575,8 +6598,9 @@
       <c r="O18" s="12"/>
       <c r="P18" s="12"/>
       <c r="Q18" s="12"/>
-    </row>
-    <row r="19" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R18" s="12"/>
+    </row>
+    <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="7">
         <v>1</v>
@@ -6607,8 +6631,9 @@
       <c r="O19" s="12"/>
       <c r="P19" s="12"/>
       <c r="Q19" s="12"/>
-    </row>
-    <row r="20" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R19" s="12"/>
+    </row>
+    <row r="20" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="7">
         <v>1</v>
@@ -6639,8 +6664,9 @@
       <c r="O20" s="12"/>
       <c r="P20" s="12"/>
       <c r="Q20" s="12"/>
-    </row>
-    <row r="21" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R20" s="12"/>
+    </row>
+    <row r="21" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="7">
         <v>1</v>
@@ -6671,8 +6697,9 @@
       <c r="O21" s="12"/>
       <c r="P21" s="12"/>
       <c r="Q21" s="12"/>
-    </row>
-    <row r="22" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R21" s="12"/>
+    </row>
+    <row r="22" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="7">
         <v>1</v>
@@ -6703,8 +6730,9 @@
       <c r="O22" s="12"/>
       <c r="P22" s="12"/>
       <c r="Q22" s="12"/>
-    </row>
-    <row r="23" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R22" s="12"/>
+    </row>
+    <row r="23" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="7">
         <v>1</v>
@@ -6735,8 +6763,9 @@
       <c r="O23" s="12"/>
       <c r="P23" s="12"/>
       <c r="Q23" s="12"/>
-    </row>
-    <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R23" s="12"/>
+    </row>
+    <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="7">
         <v>1</v>
@@ -6767,8 +6796,9 @@
       <c r="O24" s="12"/>
       <c r="P24" s="12"/>
       <c r="Q24" s="12"/>
-    </row>
-    <row r="25" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R24" s="12"/>
+    </row>
+    <row r="25" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
       <c r="B25" s="7">
         <v>1</v>
@@ -6799,6 +6829,7 @@
       <c r="O25" s="12"/>
       <c r="P25" s="12"/>
       <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="40" t="s">
@@ -6970,42 +7001,44 @@
       <c r="J37" s="20"/>
     </row>
     <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Frete</t>
+        </is>
+      </c>
+      <c r="B38" s="22"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+    </row>
+    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="25"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
-    </row>
-    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="28"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="26"/>
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="29"/>
-      <c r="C40" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
       <c r="D40" s="8"/>
       <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
+      <c r="F40" s="28"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
@@ -7013,9 +7046,9 @@
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B41" s="8"/>
+        <v>30</v>
+      </c>
+      <c r="B41" s="29"/>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
       <c r="E41" s="8"/>
@@ -7026,20 +7059,20 @@
       <c r="J41" s="8"/>
     </row>
     <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
+      <c r="A42" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="8"/>
+      <c r="J42" s="8"/>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="24" t="s">
-        <v>32</v>
-      </c>
       <c r="B43" s="26"/>
       <c r="C43" s="26"/>
       <c r="D43" s="26"/>
@@ -7051,24 +7084,24 @@
       <c r="J43" s="26"/>
     </row>
     <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
+      <c r="A44" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="26"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="26"/>
+      <c r="H44" s="26"/>
+      <c r="I44" s="26"/>
+      <c r="J44" s="26"/>
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="B45" s="28"/>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
@@ -7080,7 +7113,7 @@
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -7093,21 +7126,21 @@
       <c r="J46" s="8"/>
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="19"/>
-      <c r="B47" s="26"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
-      <c r="I47" s="26"/>
-      <c r="J47" s="26"/>
+      <c r="A47" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+      <c r="I47" s="8"/>
+      <c r="J47" s="8"/>
     </row>
     <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="24" t="s">
-        <v>33</v>
-      </c>
+      <c r="A48" s="19"/>
       <c r="B48" s="26"/>
       <c r="C48" s="26"/>
       <c r="D48" s="26"/>
@@ -7119,24 +7152,24 @@
       <c r="J48" s="26"/>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
-      <c r="J49" s="8"/>
+      <c r="A49" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="26"/>
+      <c r="J49" s="26"/>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B50" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="B50" s="28"/>
       <c r="C50" s="8"/>
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
@@ -7148,7 +7181,7 @@
     </row>
     <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -7161,20 +7194,20 @@
       <c r="J51" s="8"/>
     </row>
     <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="26"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="26"/>
-      <c r="I52" s="26"/>
-      <c r="J52" s="26"/>
+      <c r="A52" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="8"/>
+      <c r="J52" s="8"/>
     </row>
     <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="24" t="s">
-        <v>34</v>
-      </c>
       <c r="B53" s="26"/>
       <c r="C53" s="26"/>
       <c r="D53" s="26"/>
@@ -7186,24 +7219,24 @@
       <c r="J53" s="26"/>
     </row>
     <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B54" s="28"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8"/>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="8"/>
+      <c r="A54" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" s="26"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="26"/>
+      <c r="F54" s="26"/>
+      <c r="G54" s="26"/>
+      <c r="H54" s="26"/>
+      <c r="I54" s="26"/>
+      <c r="J54" s="26"/>
     </row>
     <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B55" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="B55" s="28"/>
       <c r="C55" s="8"/>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
@@ -7215,7 +7248,7 @@
     </row>
     <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -7228,20 +7261,20 @@
       <c r="J56" s="8"/>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="26"/>
-      <c r="C57" s="26"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="26"/>
-      <c r="F57" s="26"/>
-      <c r="G57" s="26"/>
-      <c r="H57" s="26"/>
-      <c r="I57" s="26"/>
-      <c r="J57" s="26"/>
+      <c r="A57" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
     </row>
     <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="24" t="s">
-        <v>35</v>
-      </c>
       <c r="B58" s="26"/>
       <c r="C58" s="26"/>
       <c r="D58" s="26"/>
@@ -7253,22 +7286,22 @@
       <c r="J58" s="26"/>
     </row>
     <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B59" s="8"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="8"/>
-      <c r="G59" s="8"/>
-      <c r="H59" s="8"/>
-      <c r="I59" s="8"/>
-      <c r="J59" s="8"/>
+      <c r="A59" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="26"/>
+      <c r="I59" s="26"/>
+      <c r="J59" s="26"/>
     </row>
     <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -7282,7 +7315,7 @@
     </row>
     <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -7295,20 +7328,20 @@
       <c r="J61" s="8"/>
     </row>
     <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="26"/>
-      <c r="E62" s="26"/>
-      <c r="F62" s="26"/>
-      <c r="G62" s="26"/>
-      <c r="H62" s="26"/>
-      <c r="I62" s="26"/>
-      <c r="J62" s="26"/>
+      <c r="A62" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B62" s="8"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="8"/>
+      <c r="H62" s="8"/>
+      <c r="I62" s="8"/>
+      <c r="J62" s="8"/>
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="24" t="s">
-        <v>36</v>
-      </c>
       <c r="B63" s="26"/>
       <c r="C63" s="26"/>
       <c r="D63" s="26"/>
@@ -7320,22 +7353,22 @@
       <c r="J63" s="26"/>
     </row>
     <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B64" s="8"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
-      <c r="I64" s="8"/>
-      <c r="J64" s="8"/>
+      <c r="A64" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B64" s="26"/>
+      <c r="C64" s="26"/>
+      <c r="D64" s="26"/>
+      <c r="E64" s="26"/>
+      <c r="F64" s="26"/>
+      <c r="G64" s="26"/>
+      <c r="H64" s="26"/>
+      <c r="I64" s="26"/>
+      <c r="J64" s="26"/>
     </row>
     <row r="65" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
@@ -7349,7 +7382,7 @@
     </row>
     <row r="66" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -7362,21 +7395,21 @@
       <c r="J66" s="8"/>
     </row>
     <row r="67" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="30"/>
-      <c r="C67" s="26"/>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="26"/>
-      <c r="G67" s="26"/>
-      <c r="H67" s="26"/>
-      <c r="I67" s="26"/>
-      <c r="J67" s="26"/>
+      <c r="A67" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="I67" s="8"/>
+      <c r="J67" s="8"/>
     </row>
     <row r="68" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="B68" s="26"/>
+      <c r="B68" s="30"/>
       <c r="C68" s="26"/>
       <c r="D68" s="26"/>
       <c r="E68" s="26"/>
@@ -7387,22 +7420,22 @@
       <c r="J68" s="26"/>
     </row>
     <row r="69" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B69" s="8"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="8"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="8"/>
-      <c r="I69" s="8"/>
-      <c r="J69" s="8"/>
+      <c r="A69" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B69" s="26"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
+      <c r="F69" s="26"/>
+      <c r="G69" s="26"/>
+      <c r="H69" s="26"/>
+      <c r="I69" s="26"/>
+      <c r="J69" s="26"/>
     </row>
     <row r="70" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
@@ -7416,7 +7449,7 @@
     </row>
     <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
@@ -7429,20 +7462,20 @@
       <c r="J71" s="8"/>
     </row>
     <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="26"/>
-      <c r="C72" s="26"/>
-      <c r="D72" s="26"/>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="26"/>
-      <c r="I72" s="26"/>
-      <c r="J72" s="26"/>
+      <c r="A72" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="8"/>
+      <c r="I72" s="8"/>
+      <c r="J72" s="8"/>
     </row>
     <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="24" t="s">
-        <v>38</v>
-      </c>
       <c r="B73" s="26"/>
       <c r="C73" s="26"/>
       <c r="D73" s="26"/>
@@ -7454,22 +7487,22 @@
       <c r="J73" s="26"/>
     </row>
     <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
-      <c r="E74" s="8"/>
-      <c r="F74" s="8"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="8"/>
-      <c r="I74" s="8"/>
-      <c r="J74" s="8"/>
+      <c r="A74" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="26"/>
+      <c r="F74" s="26"/>
+      <c r="G74" s="26"/>
+      <c r="H74" s="26"/>
+      <c r="I74" s="26"/>
+      <c r="J74" s="26"/>
     </row>
     <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -7483,7 +7516,7 @@
     </row>
     <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B76" s="8"/>
       <c r="C76" s="8"/>
@@ -7496,20 +7529,20 @@
       <c r="J76" s="8"/>
     </row>
     <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="26"/>
-      <c r="C77" s="26"/>
-      <c r="D77" s="26"/>
-      <c r="E77" s="26"/>
-      <c r="F77" s="26"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="26"/>
-      <c r="I77" s="26"/>
-      <c r="J77" s="26"/>
+      <c r="A77" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B77" s="8"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="8"/>
+      <c r="E77" s="8"/>
+      <c r="F77" s="8"/>
+      <c r="G77" s="8"/>
+      <c r="H77" s="8"/>
+      <c r="I77" s="8"/>
+      <c r="J77" s="8"/>
     </row>
     <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="24" t="s">
-        <v>39</v>
-      </c>
       <c r="B78" s="26"/>
       <c r="C78" s="26"/>
       <c r="D78" s="26"/>
@@ -7521,22 +7554,22 @@
       <c r="J78" s="26"/>
     </row>
     <row r="79" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="8"/>
-      <c r="I79" s="8"/>
-      <c r="J79" s="8"/>
+      <c r="A79" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="26"/>
+      <c r="G79" s="26"/>
+      <c r="H79" s="26"/>
+      <c r="I79" s="26"/>
+      <c r="J79" s="26"/>
     </row>
     <row r="80" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B80" s="8"/>
       <c r="C80" s="8"/>
@@ -7550,7 +7583,7 @@
     </row>
     <row r="81" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B81" s="8"/>
       <c r="C81" s="8"/>
@@ -7563,20 +7596,20 @@
       <c r="J81" s="8"/>
     </row>
     <row r="82" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="26"/>
-      <c r="C82" s="26"/>
-      <c r="D82" s="26"/>
-      <c r="E82" s="26"/>
-      <c r="F82" s="26"/>
-      <c r="G82" s="26"/>
-      <c r="H82" s="26"/>
-      <c r="I82" s="26"/>
-      <c r="J82" s="26"/>
+      <c r="A82" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B82" s="8"/>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="8"/>
+      <c r="H82" s="8"/>
+      <c r="I82" s="8"/>
+      <c r="J82" s="8"/>
     </row>
     <row r="83" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="24" t="s">
-        <v>40</v>
-      </c>
       <c r="B83" s="26"/>
       <c r="C83" s="26"/>
       <c r="D83" s="26"/>
@@ -7588,22 +7621,22 @@
       <c r="J83" s="26"/>
     </row>
     <row r="84" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="8"/>
-      <c r="I84" s="8"/>
-      <c r="J84" s="8"/>
+      <c r="A84" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B84" s="26"/>
+      <c r="C84" s="26"/>
+      <c r="D84" s="26"/>
+      <c r="E84" s="26"/>
+      <c r="F84" s="26"/>
+      <c r="G84" s="26"/>
+      <c r="H84" s="26"/>
+      <c r="I84" s="26"/>
+      <c r="J84" s="26"/>
     </row>
     <row r="85" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B85" s="8"/>
       <c r="C85" s="8"/>
@@ -7617,7 +7650,7 @@
     </row>
     <row r="86" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B86" s="8"/>
       <c r="C86" s="8"/>
@@ -7630,20 +7663,20 @@
       <c r="J86" s="8"/>
     </row>
     <row r="87" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="26"/>
-      <c r="C87" s="26"/>
-      <c r="D87" s="26"/>
-      <c r="E87" s="26"/>
-      <c r="F87" s="26"/>
-      <c r="G87" s="26"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="26"/>
-      <c r="J87" s="26"/>
+      <c r="A87" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B87" s="8"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="8"/>
+      <c r="E87" s="8"/>
+      <c r="F87" s="8"/>
+      <c r="G87" s="8"/>
+      <c r="H87" s="8"/>
+      <c r="I87" s="8"/>
+      <c r="J87" s="8"/>
     </row>
     <row r="88" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="24" t="s">
-        <v>41</v>
-      </c>
       <c r="B88" s="26"/>
       <c r="C88" s="26"/>
       <c r="D88" s="26"/>
@@ -7655,22 +7688,22 @@
       <c r="J88" s="26"/>
     </row>
     <row r="89" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
-      <c r="E89" s="8"/>
-      <c r="F89" s="8"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="8"/>
-      <c r="I89" s="8"/>
-      <c r="J89" s="8"/>
+      <c r="A89" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="B89" s="26"/>
+      <c r="C89" s="26"/>
+      <c r="D89" s="26"/>
+      <c r="E89" s="26"/>
+      <c r="F89" s="26"/>
+      <c r="G89" s="26"/>
+      <c r="H89" s="26"/>
+      <c r="I89" s="26"/>
+      <c r="J89" s="26"/>
     </row>
     <row r="90" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B90" s="8"/>
       <c r="C90" s="8"/>
@@ -7684,7 +7717,7 @@
     </row>
     <row r="91" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B91" s="8"/>
       <c r="C91" s="8"/>
@@ -7697,20 +7730,20 @@
       <c r="J91" s="8"/>
     </row>
     <row r="92" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="26"/>
-      <c r="C92" s="26"/>
-      <c r="D92" s="26"/>
-      <c r="E92" s="26"/>
-      <c r="F92" s="26"/>
-      <c r="G92" s="26"/>
-      <c r="H92" s="26"/>
-      <c r="I92" s="26"/>
-      <c r="J92" s="26"/>
+      <c r="A92" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B92" s="8"/>
+      <c r="C92" s="8"/>
+      <c r="D92" s="8"/>
+      <c r="E92" s="8"/>
+      <c r="F92" s="8"/>
+      <c r="G92" s="8"/>
+      <c r="H92" s="8"/>
+      <c r="I92" s="8"/>
+      <c r="J92" s="8"/>
     </row>
     <row r="93" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="24" t="s">
-        <v>42</v>
-      </c>
       <c r="B93" s="26"/>
       <c r="C93" s="26"/>
       <c r="D93" s="26"/>
@@ -7722,22 +7755,22 @@
       <c r="J93" s="26"/>
     </row>
     <row r="94" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
-      <c r="G94" s="8"/>
-      <c r="H94" s="8"/>
-      <c r="I94" s="8"/>
-      <c r="J94" s="8"/>
+      <c r="A94" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B94" s="26"/>
+      <c r="C94" s="26"/>
+      <c r="D94" s="26"/>
+      <c r="E94" s="26"/>
+      <c r="F94" s="26"/>
+      <c r="G94" s="26"/>
+      <c r="H94" s="26"/>
+      <c r="I94" s="26"/>
+      <c r="J94" s="26"/>
     </row>
     <row r="95" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
@@ -7751,7 +7784,7 @@
     </row>
     <row r="96" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
@@ -7764,20 +7797,20 @@
       <c r="J96" s="8"/>
     </row>
     <row r="97" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="26"/>
-      <c r="C97" s="26"/>
-      <c r="D97" s="26"/>
-      <c r="E97" s="26"/>
-      <c r="F97" s="26"/>
-      <c r="G97" s="26"/>
-      <c r="H97" s="26"/>
-      <c r="I97" s="26"/>
-      <c r="J97" s="26"/>
+      <c r="A97" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B97" s="8"/>
+      <c r="C97" s="8"/>
+      <c r="D97" s="8"/>
+      <c r="E97" s="8"/>
+      <c r="F97" s="8"/>
+      <c r="G97" s="8"/>
+      <c r="H97" s="8"/>
+      <c r="I97" s="8"/>
+      <c r="J97" s="8"/>
     </row>
     <row r="98" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="24" t="s">
-        <v>43</v>
-      </c>
       <c r="B98" s="26"/>
       <c r="C98" s="26"/>
       <c r="D98" s="26"/>
@@ -7789,22 +7822,22 @@
       <c r="J98" s="26"/>
     </row>
     <row r="99" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="8"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="8"/>
-      <c r="I99" s="8"/>
-      <c r="J99" s="8"/>
+      <c r="A99" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B99" s="26"/>
+      <c r="C99" s="26"/>
+      <c r="D99" s="26"/>
+      <c r="E99" s="26"/>
+      <c r="F99" s="26"/>
+      <c r="G99" s="26"/>
+      <c r="H99" s="26"/>
+      <c r="I99" s="26"/>
+      <c r="J99" s="26"/>
     </row>
     <row r="100" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B100" s="8"/>
       <c r="C100" s="8"/>
@@ -7818,7 +7851,7 @@
     </row>
     <row r="101" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B101" s="8"/>
       <c r="C101" s="8"/>
@@ -7831,20 +7864,20 @@
       <c r="J101" s="8"/>
     </row>
     <row r="102" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B102" s="26"/>
-      <c r="C102" s="26"/>
-      <c r="D102" s="26"/>
-      <c r="E102" s="26"/>
-      <c r="F102" s="26"/>
-      <c r="G102" s="26"/>
-      <c r="H102" s="26"/>
-      <c r="I102" s="26"/>
-      <c r="J102" s="26"/>
+      <c r="A102" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="8"/>
+      <c r="H102" s="8"/>
+      <c r="I102" s="8"/>
+      <c r="J102" s="8"/>
     </row>
     <row r="103" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="24" t="s">
-        <v>44</v>
-      </c>
       <c r="B103" s="26"/>
       <c r="C103" s="26"/>
       <c r="D103" s="26"/>
@@ -7856,22 +7889,22 @@
       <c r="J103" s="26"/>
     </row>
     <row r="104" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B104" s="8"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
-      <c r="F104" s="8"/>
-      <c r="G104" s="8"/>
-      <c r="H104" s="8"/>
-      <c r="I104" s="8"/>
-      <c r="J104" s="8"/>
+      <c r="A104" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B104" s="26"/>
+      <c r="C104" s="26"/>
+      <c r="D104" s="26"/>
+      <c r="E104" s="26"/>
+      <c r="F104" s="26"/>
+      <c r="G104" s="26"/>
+      <c r="H104" s="26"/>
+      <c r="I104" s="26"/>
+      <c r="J104" s="26"/>
     </row>
     <row r="105" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B105" s="8"/>
       <c r="C105" s="8"/>
@@ -7885,7 +7918,7 @@
     </row>
     <row r="106" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B106" s="8"/>
       <c r="C106" s="8"/>
@@ -7898,20 +7931,20 @@
       <c r="J106" s="8"/>
     </row>
     <row r="107" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B107" s="26"/>
-      <c r="C107" s="26"/>
-      <c r="D107" s="26"/>
-      <c r="E107" s="26"/>
-      <c r="F107" s="26"/>
-      <c r="G107" s="26"/>
-      <c r="H107" s="26"/>
-      <c r="I107" s="26"/>
-      <c r="J107" s="26"/>
+      <c r="A107" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B107" s="8"/>
+      <c r="C107" s="8"/>
+      <c r="D107" s="8"/>
+      <c r="E107" s="8"/>
+      <c r="F107" s="8"/>
+      <c r="G107" s="8"/>
+      <c r="H107" s="8"/>
+      <c r="I107" s="8"/>
+      <c r="J107" s="8"/>
     </row>
     <row r="108" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="24" t="s">
-        <v>45</v>
-      </c>
       <c r="B108" s="26"/>
       <c r="C108" s="26"/>
       <c r="D108" s="26"/>
@@ -7923,22 +7956,22 @@
       <c r="J108" s="26"/>
     </row>
     <row r="109" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B109" s="8"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="8"/>
-      <c r="E109" s="8"/>
-      <c r="F109" s="8"/>
-      <c r="G109" s="8"/>
-      <c r="H109" s="8"/>
-      <c r="I109" s="8"/>
-      <c r="J109" s="8"/>
+      <c r="A109" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="B109" s="26"/>
+      <c r="C109" s="26"/>
+      <c r="D109" s="26"/>
+      <c r="E109" s="26"/>
+      <c r="F109" s="26"/>
+      <c r="G109" s="26"/>
+      <c r="H109" s="26"/>
+      <c r="I109" s="26"/>
+      <c r="J109" s="26"/>
     </row>
     <row r="110" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B110" s="8"/>
       <c r="C110" s="8"/>
@@ -7952,7 +7985,7 @@
     </row>
     <row r="111" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B111" s="8"/>
       <c r="C111" s="8"/>
@@ -7965,20 +7998,20 @@
       <c r="J111" s="8"/>
     </row>
     <row r="112" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="26"/>
-      <c r="C112" s="26"/>
-      <c r="D112" s="26"/>
-      <c r="E112" s="26"/>
-      <c r="F112" s="26"/>
-      <c r="G112" s="26"/>
-      <c r="H112" s="26"/>
-      <c r="I112" s="26"/>
-      <c r="J112" s="26"/>
+      <c r="A112" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B112" s="8"/>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8"/>
+      <c r="G112" s="8"/>
+      <c r="H112" s="8"/>
+      <c r="I112" s="8"/>
+      <c r="J112" s="8"/>
     </row>
     <row r="113" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="24" t="s">
-        <v>46</v>
-      </c>
       <c r="B113" s="26"/>
       <c r="C113" s="26"/>
       <c r="D113" s="26"/>
@@ -7990,22 +8023,22 @@
       <c r="J113" s="26"/>
     </row>
     <row r="114" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B114" s="8"/>
-      <c r="C114" s="8"/>
-      <c r="D114" s="8"/>
-      <c r="E114" s="8"/>
-      <c r="F114" s="8"/>
-      <c r="G114" s="8"/>
-      <c r="H114" s="8"/>
-      <c r="I114" s="8"/>
-      <c r="J114" s="8"/>
+      <c r="A114" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B114" s="26"/>
+      <c r="C114" s="26"/>
+      <c r="D114" s="26"/>
+      <c r="E114" s="26"/>
+      <c r="F114" s="26"/>
+      <c r="G114" s="26"/>
+      <c r="H114" s="26"/>
+      <c r="I114" s="26"/>
+      <c r="J114" s="26"/>
     </row>
     <row r="115" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B115" s="8"/>
       <c r="C115" s="8"/>
@@ -8019,7 +8052,7 @@
     </row>
     <row r="116" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B116" s="8"/>
       <c r="C116" s="8"/>
@@ -8032,20 +8065,20 @@
       <c r="J116" s="8"/>
     </row>
     <row r="117" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="26"/>
-      <c r="C117" s="26"/>
-      <c r="D117" s="26"/>
-      <c r="E117" s="26"/>
-      <c r="F117" s="26"/>
-      <c r="G117" s="26"/>
-      <c r="H117" s="26"/>
-      <c r="I117" s="26"/>
-      <c r="J117" s="26"/>
+      <c r="A117" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B117" s="8"/>
+      <c r="C117" s="8"/>
+      <c r="D117" s="8"/>
+      <c r="E117" s="8"/>
+      <c r="F117" s="8"/>
+      <c r="G117" s="8"/>
+      <c r="H117" s="8"/>
+      <c r="I117" s="8"/>
+      <c r="J117" s="8"/>
     </row>
     <row r="118" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="24" t="s">
-        <v>47</v>
-      </c>
       <c r="B118" s="26"/>
       <c r="C118" s="26"/>
       <c r="D118" s="26"/>
@@ -8057,22 +8090,22 @@
       <c r="J118" s="26"/>
     </row>
     <row r="119" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B119" s="8"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="8"/>
-      <c r="E119" s="8"/>
-      <c r="F119" s="8"/>
-      <c r="G119" s="8"/>
-      <c r="H119" s="8"/>
-      <c r="I119" s="8"/>
-      <c r="J119" s="8"/>
+      <c r="A119" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B119" s="26"/>
+      <c r="C119" s="26"/>
+      <c r="D119" s="26"/>
+      <c r="E119" s="26"/>
+      <c r="F119" s="26"/>
+      <c r="G119" s="26"/>
+      <c r="H119" s="26"/>
+      <c r="I119" s="26"/>
+      <c r="J119" s="26"/>
     </row>
     <row r="120" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B120" s="8"/>
       <c r="C120" s="8"/>
@@ -8086,7 +8119,7 @@
     </row>
     <row r="121" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B121" s="8"/>
       <c r="C121" s="8"/>
@@ -8099,20 +8132,20 @@
       <c r="J121" s="8"/>
     </row>
     <row r="122" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B122" s="26"/>
-      <c r="C122" s="26"/>
-      <c r="D122" s="26"/>
-      <c r="E122" s="26"/>
-      <c r="F122" s="26"/>
-      <c r="G122" s="26"/>
-      <c r="H122" s="26"/>
-      <c r="I122" s="26"/>
-      <c r="J122" s="26"/>
+      <c r="A122" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B122" s="8"/>
+      <c r="C122" s="8"/>
+      <c r="D122" s="8"/>
+      <c r="E122" s="8"/>
+      <c r="F122" s="8"/>
+      <c r="G122" s="8"/>
+      <c r="H122" s="8"/>
+      <c r="I122" s="8"/>
+      <c r="J122" s="8"/>
     </row>
     <row r="123" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="24" t="s">
-        <v>48</v>
-      </c>
       <c r="B123" s="26"/>
       <c r="C123" s="26"/>
       <c r="D123" s="26"/>
@@ -8124,22 +8157,22 @@
       <c r="J123" s="26"/>
     </row>
     <row r="124" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B124" s="8"/>
-      <c r="C124" s="8"/>
-      <c r="D124" s="8"/>
-      <c r="E124" s="8"/>
-      <c r="F124" s="8"/>
-      <c r="G124" s="8"/>
-      <c r="H124" s="8"/>
-      <c r="I124" s="8"/>
-      <c r="J124" s="8"/>
+      <c r="A124" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B124" s="26"/>
+      <c r="C124" s="26"/>
+      <c r="D124" s="26"/>
+      <c r="E124" s="26"/>
+      <c r="F124" s="26"/>
+      <c r="G124" s="26"/>
+      <c r="H124" s="26"/>
+      <c r="I124" s="26"/>
+      <c r="J124" s="26"/>
     </row>
     <row r="125" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B125" s="8"/>
       <c r="C125" s="8"/>
@@ -8153,7 +8186,7 @@
     </row>
     <row r="126" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B126" s="8"/>
       <c r="C126" s="8"/>
@@ -8166,20 +8199,20 @@
       <c r="J126" s="8"/>
     </row>
     <row r="127" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B127" s="26"/>
-      <c r="C127" s="26"/>
-      <c r="D127" s="26"/>
-      <c r="E127" s="26"/>
-      <c r="F127" s="26"/>
-      <c r="G127" s="26"/>
-      <c r="H127" s="26"/>
-      <c r="I127" s="26"/>
-      <c r="J127" s="26"/>
+      <c r="A127" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B127" s="8"/>
+      <c r="C127" s="8"/>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8"/>
+      <c r="F127" s="8"/>
+      <c r="G127" s="8"/>
+      <c r="H127" s="8"/>
+      <c r="I127" s="8"/>
+      <c r="J127" s="8"/>
     </row>
     <row r="128" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="24" t="s">
-        <v>49</v>
-      </c>
       <c r="B128" s="26"/>
       <c r="C128" s="26"/>
       <c r="D128" s="26"/>
@@ -8191,22 +8224,22 @@
       <c r="J128" s="26"/>
     </row>
     <row r="129" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B129" s="8"/>
-      <c r="C129" s="8"/>
-      <c r="D129" s="8"/>
-      <c r="E129" s="8"/>
-      <c r="F129" s="8"/>
-      <c r="G129" s="8"/>
-      <c r="H129" s="8"/>
-      <c r="I129" s="8"/>
-      <c r="J129" s="8"/>
+      <c r="A129" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B129" s="26"/>
+      <c r="C129" s="26"/>
+      <c r="D129" s="26"/>
+      <c r="E129" s="26"/>
+      <c r="F129" s="26"/>
+      <c r="G129" s="26"/>
+      <c r="H129" s="26"/>
+      <c r="I129" s="26"/>
+      <c r="J129" s="26"/>
     </row>
     <row r="130" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B130" s="8"/>
       <c r="C130" s="8"/>
@@ -8220,7 +8253,7 @@
     </row>
     <row r="131" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B131" s="8"/>
       <c r="C131" s="8"/>
@@ -8233,20 +8266,20 @@
       <c r="J131" s="8"/>
     </row>
     <row r="132" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B132" s="26"/>
-      <c r="C132" s="26"/>
-      <c r="D132" s="26"/>
-      <c r="E132" s="26"/>
-      <c r="F132" s="26"/>
-      <c r="G132" s="26"/>
-      <c r="H132" s="26"/>
-      <c r="I132" s="26"/>
-      <c r="J132" s="26"/>
+      <c r="A132" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B132" s="8"/>
+      <c r="C132" s="8"/>
+      <c r="D132" s="8"/>
+      <c r="E132" s="8"/>
+      <c r="F132" s="8"/>
+      <c r="G132" s="8"/>
+      <c r="H132" s="8"/>
+      <c r="I132" s="8"/>
+      <c r="J132" s="8"/>
     </row>
     <row r="133" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="24" t="s">
-        <v>50</v>
-      </c>
       <c r="B133" s="26"/>
       <c r="C133" s="26"/>
       <c r="D133" s="26"/>
@@ -8258,22 +8291,22 @@
       <c r="J133" s="26"/>
     </row>
     <row r="134" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B134" s="8"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="8"/>
-      <c r="E134" s="8"/>
-      <c r="F134" s="8"/>
-      <c r="G134" s="8"/>
-      <c r="H134" s="8"/>
-      <c r="I134" s="8"/>
-      <c r="J134" s="8"/>
+      <c r="A134" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B134" s="26"/>
+      <c r="C134" s="26"/>
+      <c r="D134" s="26"/>
+      <c r="E134" s="26"/>
+      <c r="F134" s="26"/>
+      <c r="G134" s="26"/>
+      <c r="H134" s="26"/>
+      <c r="I134" s="26"/>
+      <c r="J134" s="26"/>
     </row>
     <row r="135" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B135" s="8"/>
       <c r="C135" s="8"/>
@@ -8287,7 +8320,7 @@
     </row>
     <row r="136" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B136" s="8"/>
       <c r="C136" s="8"/>
@@ -8300,20 +8333,20 @@
       <c r="J136" s="8"/>
     </row>
     <row r="137" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B137" s="26"/>
-      <c r="C137" s="26"/>
-      <c r="D137" s="26"/>
-      <c r="E137" s="26"/>
-      <c r="F137" s="26"/>
-      <c r="G137" s="26"/>
-      <c r="H137" s="26"/>
-      <c r="I137" s="26"/>
-      <c r="J137" s="26"/>
+      <c r="A137" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B137" s="8"/>
+      <c r="C137" s="8"/>
+      <c r="D137" s="8"/>
+      <c r="E137" s="8"/>
+      <c r="F137" s="8"/>
+      <c r="G137" s="8"/>
+      <c r="H137" s="8"/>
+      <c r="I137" s="8"/>
+      <c r="J137" s="8"/>
     </row>
     <row r="138" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="24" t="s">
-        <v>51</v>
-      </c>
       <c r="B138" s="26"/>
       <c r="C138" s="26"/>
       <c r="D138" s="26"/>
@@ -8325,22 +8358,22 @@
       <c r="J138" s="26"/>
     </row>
     <row r="139" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B139" s="8"/>
-      <c r="C139" s="8"/>
-      <c r="D139" s="8"/>
-      <c r="E139" s="8"/>
-      <c r="F139" s="8"/>
-      <c r="G139" s="8"/>
-      <c r="H139" s="8"/>
-      <c r="I139" s="8"/>
-      <c r="J139" s="8"/>
+      <c r="A139" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B139" s="26"/>
+      <c r="C139" s="26"/>
+      <c r="D139" s="26"/>
+      <c r="E139" s="26"/>
+      <c r="F139" s="26"/>
+      <c r="G139" s="26"/>
+      <c r="H139" s="26"/>
+      <c r="I139" s="26"/>
+      <c r="J139" s="26"/>
     </row>
     <row r="140" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B140" s="8"/>
       <c r="C140" s="8"/>
@@ -8354,7 +8387,7 @@
     </row>
     <row r="141" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B141" s="8"/>
       <c r="C141" s="8"/>
@@ -8367,20 +8400,20 @@
       <c r="J141" s="8"/>
     </row>
     <row r="142" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B142" s="26"/>
-      <c r="C142" s="26"/>
-      <c r="D142" s="26"/>
-      <c r="E142" s="26"/>
-      <c r="F142" s="26"/>
-      <c r="G142" s="26"/>
-      <c r="H142" s="26"/>
-      <c r="I142" s="26"/>
-      <c r="J142" s="26"/>
+      <c r="A142" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B142" s="8"/>
+      <c r="C142" s="8"/>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8"/>
+      <c r="G142" s="8"/>
+      <c r="H142" s="8"/>
+      <c r="I142" s="8"/>
+      <c r="J142" s="8"/>
     </row>
     <row r="143" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="24" t="s">
-        <v>52</v>
-      </c>
       <c r="B143" s="26"/>
       <c r="C143" s="26"/>
       <c r="D143" s="26"/>
@@ -8392,22 +8425,22 @@
       <c r="J143" s="26"/>
     </row>
     <row r="144" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B144" s="8"/>
-      <c r="C144" s="8"/>
-      <c r="D144" s="8"/>
-      <c r="E144" s="8"/>
-      <c r="F144" s="8"/>
-      <c r="G144" s="8"/>
-      <c r="H144" s="8"/>
-      <c r="I144" s="8"/>
-      <c r="J144" s="8"/>
+      <c r="A144" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B144" s="26"/>
+      <c r="C144" s="26"/>
+      <c r="D144" s="26"/>
+      <c r="E144" s="26"/>
+      <c r="F144" s="26"/>
+      <c r="G144" s="26"/>
+      <c r="H144" s="26"/>
+      <c r="I144" s="26"/>
+      <c r="J144" s="26"/>
     </row>
     <row r="145" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B145" s="8"/>
       <c r="C145" s="8"/>
@@ -8421,7 +8454,7 @@
     </row>
     <row r="146" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B146" s="8"/>
       <c r="C146" s="8"/>
@@ -8434,20 +8467,20 @@
       <c r="J146" s="8"/>
     </row>
     <row r="147" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B147" s="26"/>
-      <c r="C147" s="26"/>
-      <c r="D147" s="26"/>
-      <c r="E147" s="26"/>
-      <c r="F147" s="26"/>
-      <c r="G147" s="26"/>
-      <c r="H147" s="26"/>
-      <c r="I147" s="26"/>
-      <c r="J147" s="26"/>
+      <c r="A147" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B147" s="8"/>
+      <c r="C147" s="8"/>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8"/>
+      <c r="F147" s="8"/>
+      <c r="G147" s="8"/>
+      <c r="H147" s="8"/>
+      <c r="I147" s="8"/>
+      <c r="J147" s="8"/>
     </row>
     <row r="148" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="24" t="s">
-        <v>53</v>
-      </c>
       <c r="B148" s="26"/>
       <c r="C148" s="26"/>
       <c r="D148" s="26"/>
@@ -8459,22 +8492,22 @@
       <c r="J148" s="26"/>
     </row>
     <row r="149" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B149" s="8"/>
-      <c r="C149" s="8"/>
-      <c r="D149" s="8"/>
-      <c r="E149" s="8"/>
-      <c r="F149" s="8"/>
-      <c r="G149" s="8"/>
-      <c r="H149" s="8"/>
-      <c r="I149" s="8"/>
-      <c r="J149" s="8"/>
+      <c r="A149" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B149" s="26"/>
+      <c r="C149" s="26"/>
+      <c r="D149" s="26"/>
+      <c r="E149" s="26"/>
+      <c r="F149" s="26"/>
+      <c r="G149" s="26"/>
+      <c r="H149" s="26"/>
+      <c r="I149" s="26"/>
+      <c r="J149" s="26"/>
     </row>
     <row r="150" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B150" s="8"/>
       <c r="C150" s="8"/>
@@ -8488,7 +8521,7 @@
     </row>
     <row r="151" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B151" s="8"/>
       <c r="C151" s="8"/>
@@ -8501,20 +8534,20 @@
       <c r="J151" s="8"/>
     </row>
     <row r="152" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B152" s="26"/>
-      <c r="C152" s="26"/>
-      <c r="D152" s="26"/>
-      <c r="E152" s="26"/>
-      <c r="F152" s="26"/>
-      <c r="G152" s="26"/>
-      <c r="H152" s="26"/>
-      <c r="I152" s="26"/>
-      <c r="J152" s="26"/>
+      <c r="A152" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B152" s="8"/>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="8"/>
+      <c r="H152" s="8"/>
+      <c r="I152" s="8"/>
+      <c r="J152" s="8"/>
     </row>
     <row r="153" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="24" t="s">
-        <v>54</v>
-      </c>
       <c r="B153" s="26"/>
       <c r="C153" s="26"/>
       <c r="D153" s="26"/>
@@ -8526,22 +8559,22 @@
       <c r="J153" s="26"/>
     </row>
     <row r="154" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B154" s="8"/>
-      <c r="C154" s="8"/>
-      <c r="D154" s="8"/>
-      <c r="E154" s="8"/>
-      <c r="F154" s="8"/>
-      <c r="G154" s="8"/>
-      <c r="H154" s="8"/>
-      <c r="I154" s="8"/>
-      <c r="J154" s="8"/>
+      <c r="A154" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B154" s="26"/>
+      <c r="C154" s="26"/>
+      <c r="D154" s="26"/>
+      <c r="E154" s="26"/>
+      <c r="F154" s="26"/>
+      <c r="G154" s="26"/>
+      <c r="H154" s="26"/>
+      <c r="I154" s="26"/>
+      <c r="J154" s="26"/>
     </row>
     <row r="155" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B155" s="8"/>
       <c r="C155" s="8"/>
@@ -8555,7 +8588,7 @@
     </row>
     <row r="156" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B156" s="8"/>
       <c r="C156" s="8"/>
@@ -8568,20 +8601,20 @@
       <c r="J156" s="8"/>
     </row>
     <row r="157" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B157" s="26"/>
-      <c r="C157" s="26"/>
-      <c r="D157" s="26"/>
-      <c r="E157" s="26"/>
-      <c r="F157" s="26"/>
-      <c r="G157" s="26"/>
-      <c r="H157" s="26"/>
-      <c r="I157" s="26"/>
-      <c r="J157" s="26"/>
+      <c r="A157" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B157" s="8"/>
+      <c r="C157" s="8"/>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8"/>
+      <c r="F157" s="8"/>
+      <c r="G157" s="8"/>
+      <c r="H157" s="8"/>
+      <c r="I157" s="8"/>
+      <c r="J157" s="8"/>
     </row>
     <row r="158" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="24" t="s">
-        <v>55</v>
-      </c>
       <c r="B158" s="26"/>
       <c r="C158" s="26"/>
       <c r="D158" s="26"/>
@@ -8593,22 +8626,22 @@
       <c r="J158" s="26"/>
     </row>
     <row r="159" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B159" s="8"/>
-      <c r="C159" s="8"/>
-      <c r="D159" s="8"/>
-      <c r="E159" s="8"/>
-      <c r="F159" s="8"/>
-      <c r="G159" s="8"/>
-      <c r="H159" s="8"/>
-      <c r="I159" s="8"/>
-      <c r="J159" s="8"/>
+      <c r="A159" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B159" s="26"/>
+      <c r="C159" s="26"/>
+      <c r="D159" s="26"/>
+      <c r="E159" s="26"/>
+      <c r="F159" s="26"/>
+      <c r="G159" s="26"/>
+      <c r="H159" s="26"/>
+      <c r="I159" s="26"/>
+      <c r="J159" s="26"/>
     </row>
     <row r="160" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B160" s="8"/>
       <c r="C160" s="8"/>
@@ -8622,7 +8655,7 @@
     </row>
     <row r="161" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B161" s="8"/>
       <c r="C161" s="8"/>
@@ -8635,20 +8668,20 @@
       <c r="J161" s="8"/>
     </row>
     <row r="162" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B162" s="26"/>
-      <c r="C162" s="26"/>
-      <c r="D162" s="26"/>
-      <c r="E162" s="26"/>
-      <c r="F162" s="26"/>
-      <c r="G162" s="26"/>
-      <c r="H162" s="26"/>
-      <c r="I162" s="26"/>
-      <c r="J162" s="26"/>
+      <c r="A162" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B162" s="8"/>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="8"/>
+      <c r="G162" s="8"/>
+      <c r="H162" s="8"/>
+      <c r="I162" s="8"/>
+      <c r="J162" s="8"/>
     </row>
     <row r="163" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="24" t="s">
-        <v>56</v>
-      </c>
       <c r="B163" s="26"/>
       <c r="C163" s="26"/>
       <c r="D163" s="26"/>
@@ -8660,22 +8693,22 @@
       <c r="J163" s="26"/>
     </row>
     <row r="164" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B164" s="8"/>
-      <c r="C164" s="8"/>
-      <c r="D164" s="8"/>
-      <c r="E164" s="8"/>
-      <c r="F164" s="8"/>
-      <c r="G164" s="8"/>
-      <c r="H164" s="8"/>
-      <c r="I164" s="8"/>
-      <c r="J164" s="8"/>
+      <c r="A164" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B164" s="26"/>
+      <c r="C164" s="26"/>
+      <c r="D164" s="26"/>
+      <c r="E164" s="26"/>
+      <c r="F164" s="26"/>
+      <c r="G164" s="26"/>
+      <c r="H164" s="26"/>
+      <c r="I164" s="26"/>
+      <c r="J164" s="26"/>
     </row>
     <row r="165" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B165" s="8"/>
       <c r="C165" s="8"/>
@@ -8689,7 +8722,7 @@
     </row>
     <row r="166" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B166" s="8"/>
       <c r="C166" s="8"/>
@@ -8702,20 +8735,20 @@
       <c r="J166" s="8"/>
     </row>
     <row r="167" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B167" s="26"/>
-      <c r="C167" s="26"/>
-      <c r="D167" s="26"/>
-      <c r="E167" s="26"/>
-      <c r="F167" s="26"/>
-      <c r="G167" s="26"/>
-      <c r="H167" s="26"/>
-      <c r="I167" s="26"/>
-      <c r="J167" s="26"/>
+      <c r="A167" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B167" s="8"/>
+      <c r="C167" s="8"/>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8"/>
+      <c r="F167" s="8"/>
+      <c r="G167" s="8"/>
+      <c r="H167" s="8"/>
+      <c r="I167" s="8"/>
+      <c r="J167" s="8"/>
     </row>
     <row r="168" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="24" t="s">
-        <v>57</v>
-      </c>
       <c r="B168" s="26"/>
       <c r="C168" s="26"/>
       <c r="D168" s="26"/>
@@ -8727,22 +8760,22 @@
       <c r="J168" s="26"/>
     </row>
     <row r="169" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A169" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B169" s="8"/>
-      <c r="C169" s="8"/>
-      <c r="D169" s="8"/>
-      <c r="E169" s="8"/>
-      <c r="F169" s="8"/>
-      <c r="G169" s="8"/>
-      <c r="H169" s="8"/>
-      <c r="I169" s="8"/>
-      <c r="J169" s="8"/>
+      <c r="A169" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B169" s="26"/>
+      <c r="C169" s="26"/>
+      <c r="D169" s="26"/>
+      <c r="E169" s="26"/>
+      <c r="F169" s="26"/>
+      <c r="G169" s="26"/>
+      <c r="H169" s="26"/>
+      <c r="I169" s="26"/>
+      <c r="J169" s="26"/>
     </row>
     <row r="170" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B170" s="8"/>
       <c r="C170" s="8"/>
@@ -8756,7 +8789,7 @@
     </row>
     <row r="171" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B171" s="8"/>
       <c r="C171" s="8"/>
@@ -8769,16 +8802,18 @@
       <c r="J171" s="8"/>
     </row>
     <row r="172" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="19"/>
-      <c r="B172" s="19"/>
-      <c r="C172" s="20"/>
-      <c r="D172" s="20"/>
-      <c r="E172" s="20"/>
-      <c r="F172" s="20"/>
-      <c r="G172" s="19"/>
-      <c r="H172" s="20"/>
-      <c r="I172" s="20"/>
-      <c r="J172" s="20"/>
+      <c r="A172" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B172" s="8"/>
+      <c r="C172" s="8"/>
+      <c r="D172" s="8"/>
+      <c r="E172" s="8"/>
+      <c r="F172" s="8"/>
+      <c r="G172" s="8"/>
+      <c r="H172" s="8"/>
+      <c r="I172" s="8"/>
+      <c r="J172" s="8"/>
     </row>
     <row r="173" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="19"/>
@@ -14911,6 +14946,18 @@
       <c r="H683" s="20"/>
       <c r="I683" s="20"/>
       <c r="J683" s="20"/>
+    </row>
+    <row r="684" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A684" s="19"/>
+      <c r="B684" s="19"/>
+      <c r="C684" s="20"/>
+      <c r="D684" s="20"/>
+      <c r="E684" s="20"/>
+      <c r="F684" s="20"/>
+      <c r="G684" s="19"/>
+      <c r="H684" s="20"/>
+      <c r="I684" s="20"/>
+      <c r="J684" s="20"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="dBSKl+jny5LNm2j0K1MNTM4bqL91CvFFLDcfyHZNvPkQBIAxnXocZWIBOX0bmcnnZZZs+S64vusphakmBDKfgA==" saltValue="u8+rUr4TARUHghHw94+4zw==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0"/>
@@ -14934,7 +14981,7 @@
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>LISTAS!$A$2:$A$28</xm:f>
@@ -14998,6 +15045,15 @@
           </x14:formula2>
           <xm:sqref>Q2:Q25</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000008000000}">
+          <x14:formula1>
+            <xm:f>LISTAS!$H$2:$H$3</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>B38</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -15026,14 +15082,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G1409"/>
+  <dimension ref="A1:H1409"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="38" style="31" customWidth="1"/>
     <col min="5" max="7" width="40" style="31" customWidth="1"/>
+    <col min="8" max="8" width="20" style="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="34" t="s">
         <v>23</v>
       </c>
@@ -15055,8 +15112,13 @@
       <c r="G1" s="34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="34" t="inlineStr">
+        <is>
+          <t>FRETE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>61</v>
       </c>
@@ -15078,8 +15140,13 @@
       <c r="G2" s="33" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="33" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>127</v>
       </c>
@@ -15100,6 +15167,11 @@
       </c>
       <c r="G3" s="33" t="s">
         <v>129</v>
+      </c>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>FOB</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>